<commit_message>
Update sticker generation script and add bug documentation
- Modified `run_sheet.py` to change order details from Grove Street to Parkleigh Road, reflecting new address data.
- Updated `sheet.pdf` to match the new address format and details.
- Added a new icon asset for the house banner design.
- Introduced `BUGS.md` to document user testing issues and UX concerns for the Order Machine plugin, capturing observed bugs and expected behaviors.

This commit enhances the sticker generation process and establishes a framework for tracking bugs and UX issues during testing.
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2 old.xlsx
+++ b/stikerts/StickerBinStickersCosts v2 old.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD330459-99FD-4F8C-892E-18FE9514D80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDEBF36C-253C-47E0-8CB4-1581F2C84EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -962,11 +962,11 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1814,12 +1814,12 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A46" s="52" t="s">
+      <c r="A46" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="B46" s="52"/>
-      <c r="C46" s="52"/>
-      <c r="D46" s="52"/>
+      <c r="B46" s="54"/>
+      <c r="C46" s="54"/>
+      <c r="D46" s="54"/>
     </row>
     <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="23" t="s">
@@ -1827,12 +1827,12 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A49" s="52" t="s">
+      <c r="A49" s="54" t="s">
         <v>47</v>
       </c>
-      <c r="B49" s="52"/>
-      <c r="C49" s="52"/>
-      <c r="D49" s="52"/>
+      <c r="B49" s="54"/>
+      <c r="C49" s="54"/>
+      <c r="D49" s="54"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="17" t="s">
@@ -1894,12 +1894,12 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="52" t="s">
+      <c r="A59" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="B59" s="52"/>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
+      <c r="B59" s="54"/>
+      <c r="C59" s="54"/>
+      <c r="D59" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2411,11 +2411,11 @@
       </c>
     </row>
     <row r="56" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="53" t="s">
+      <c r="A56" s="55" t="s">
         <v>127</v>
       </c>
-      <c r="B56" s="53"/>
-      <c r="C56" s="53"/>
+      <c r="B56" s="55"/>
+      <c r="C56" s="55"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="37"/>
@@ -2508,11 +2508,11 @@
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="54" t="s">
+      <c r="A71" s="56" t="s">
         <v>137</v>
       </c>
-      <c r="B71" s="54"/>
-      <c r="C71" s="54"/>
+      <c r="B71" s="56"/>
+      <c r="C71" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2541,12 +2541,12 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
@@ -2568,7 +2568,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="52" t="s">
         <v>197</v>
       </c>
       <c r="B6" s="18">
@@ -2582,7 +2582,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="56" t="s">
+      <c r="A7" s="53" t="s">
         <v>198</v>
       </c>
       <c r="B7" s="18">
@@ -2638,12 +2638,12 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="52" t="s">
+      <c r="A13" s="54" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="52"/>
-      <c r="D13" s="52"/>
+      <c r="B13" s="54"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">

</xml_diff>